<commit_message>
Split J31122501 into hand-trimmed and machine-trimmed preparation rows
Owner decision: both preparations carry complete release panels (potency +
micro + chem each), so the batch is split into two register rows matching
the owner's own Batch Assignments naming:
- J31122501 (hand-trimmed): 100-2-K-26 THC 19.84, 231-0394-26 micro
  (TAMC 850), 1628-2026 chem — experimental processing-mode comparison,
  no CoQ issued
- J31122501 (machine-trimmed): 100-3-K-26 THC 21.84, 230-0393-26 micro
  (TAMC 1900), 1625-2026 chem — released preparation, CoQ-PP-2026-0054
Product code synced to owner spec ladder (J31_THC21.5:CBD1, Spec II,
18.84-24.25%). Register/dossier CSVs regenerated programmatically from
consolidated.json (15 stale cells from earlier renditions corrected in the
process); published Sheets verified cell-by-cell against the CSV via export
diff (0 differences).

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DyBhj47i7bhaCyNMB1iwdv
</commit_message>
<xml_diff>
--- a/deliverables/qc_register/PP_QC_eCoA_Master_Register.xlsx
+++ b/deliverables/qc_register/PP_QC_eCoA_Master_Register.xlsx
@@ -32912,7 +32912,7 @@
       </c>
       <c r="B236" s="6" t="inlineStr">
         <is>
-          <t>J31122501</t>
+          <t>J31122501 (hand-trimmed)</t>
         </is>
       </c>
       <c r="C236" s="7" t="inlineStr">
@@ -33063,22 +33063,22 @@
       <c r="D237" s="10" t="inlineStr"/>
       <c r="E237" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>19.84</t>
         </is>
       </c>
       <c r="F237" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>18.84–24.25%</t>
         </is>
       </c>
       <c r="G237" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>&lt;LOQ</t>
         </is>
       </c>
       <c r="H237" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>&lt;LOQ</t>
         </is>
       </c>
       <c r="I237" s="9" t="inlineStr">
@@ -33108,12 +33108,12 @@
       </c>
       <c r="N237" s="9" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>/</t>
         </is>
       </c>
       <c r="O237" s="9" t="inlineStr">
         <is>
-          <t>840</t>
+          <t>/</t>
         </is>
       </c>
       <c r="P237" s="9" t="inlineStr">
@@ -33123,12 +33123,12 @@
       </c>
       <c r="Q237" s="9" t="inlineStr">
         <is>
-          <t>Одговара</t>
+          <t>/</t>
         </is>
       </c>
       <c r="R237" s="9" t="inlineStr">
         <is>
-          <t>Одговара</t>
+          <t>/</t>
         </is>
       </c>
       <c r="S237" s="9" t="inlineStr">
@@ -33173,17 +33173,17 @@
       </c>
       <c r="AA237" s="9" t="inlineStr">
         <is>
-          <t>230-0393-26</t>
+          <t>100-2-K-26</t>
         </is>
       </c>
       <c r="AB237" s="9" t="inlineStr">
         <is>
-          <t>07.04.2026</t>
+          <t>09.04.2026</t>
         </is>
       </c>
       <c r="AC237" s="10" t="inlineStr">
         <is>
-          <t>IPH — Institute of Public Health (microbiology)</t>
+          <t>Farmahem</t>
         </is>
       </c>
       <c r="AD237" s="11" t="inlineStr">
@@ -33199,7 +33199,7 @@
       <c r="D238" s="10" t="inlineStr"/>
       <c r="E238" s="9" t="inlineStr">
         <is>
-          <t>21.84</t>
+          <t>/</t>
         </is>
       </c>
       <c r="F238" s="9" t="inlineStr">
@@ -33209,12 +33209,12 @@
       </c>
       <c r="G238" s="9" t="inlineStr">
         <is>
-          <t>&lt;LOQ</t>
+          <t>/</t>
         </is>
       </c>
       <c r="H238" s="9" t="inlineStr">
         <is>
-          <t>&lt;LOQ</t>
+          <t>/</t>
         </is>
       </c>
       <c r="I238" s="9" t="inlineStr">
@@ -33269,57 +33269,57 @@
       </c>
       <c r="S238" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>2,5</t>
         </is>
       </c>
       <c r="T238" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>н.д.</t>
         </is>
       </c>
       <c r="U238" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>н.д.</t>
         </is>
       </c>
       <c r="V238" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>н.д.</t>
         </is>
       </c>
       <c r="W238" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>н.д.</t>
         </is>
       </c>
       <c r="X238" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>н.д.</t>
         </is>
       </c>
       <c r="Y238" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>н.д.</t>
         </is>
       </c>
       <c r="Z238" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>н.д.</t>
         </is>
       </c>
       <c r="AA238" s="9" t="inlineStr">
         <is>
-          <t>100-3-K-26</t>
+          <t>1628-2026</t>
         </is>
       </c>
       <c r="AB238" s="9" t="inlineStr">
         <is>
-          <t>09.04.2026</t>
+          <t>23.04.2026</t>
         </is>
       </c>
       <c r="AC238" s="10" t="inlineStr">
         <is>
-          <t>Farmahem</t>
+          <t>IPH — Institute of Public Health (chemistry)</t>
         </is>
       </c>
       <c r="AD238" s="11" t="inlineStr">
@@ -33329,13 +33329,27 @@
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="9" t="inlineStr"/>
-      <c r="B239" s="12" t="inlineStr"/>
-      <c r="C239" s="9" t="inlineStr"/>
-      <c r="D239" s="10" t="inlineStr"/>
+      <c r="A239" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="B239" s="6" t="inlineStr">
+        <is>
+          <t>J31122501 (machine-trimmed)</t>
+        </is>
+      </c>
+      <c r="C239" s="7" t="inlineStr">
+        <is>
+          <t>P060262</t>
+        </is>
+      </c>
+      <c r="D239" s="8" t="inlineStr">
+        <is>
+          <t>Jokerz 31</t>
+        </is>
+      </c>
       <c r="E239" s="9" t="inlineStr">
         <is>
-          <t>19.84</t>
+          <t>/</t>
         </is>
       </c>
       <c r="F239" s="9" t="inlineStr">
@@ -33345,12 +33359,12 @@
       </c>
       <c r="G239" s="9" t="inlineStr">
         <is>
-          <t>&lt;LOQ</t>
+          <t>/</t>
         </is>
       </c>
       <c r="H239" s="9" t="inlineStr">
         <is>
-          <t>&lt;LOQ</t>
+          <t>/</t>
         </is>
       </c>
       <c r="I239" s="9" t="inlineStr">
@@ -33380,12 +33394,12 @@
       </c>
       <c r="N239" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="O239" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>840</t>
         </is>
       </c>
       <c r="P239" s="9" t="inlineStr">
@@ -33395,12 +33409,12 @@
       </c>
       <c r="Q239" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>Одговара</t>
         </is>
       </c>
       <c r="R239" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>Одговара</t>
         </is>
       </c>
       <c r="S239" s="9" t="inlineStr">
@@ -33445,17 +33459,17 @@
       </c>
       <c r="AA239" s="9" t="inlineStr">
         <is>
-          <t>100-2-K-26</t>
+          <t>230-0393-26</t>
         </is>
       </c>
       <c r="AB239" s="9" t="inlineStr">
         <is>
-          <t>09.04.2026</t>
+          <t>07.04.2026</t>
         </is>
       </c>
       <c r="AC239" s="10" t="inlineStr">
         <is>
-          <t>Farmahem</t>
+          <t>IPH — Institute of Public Health (microbiology)</t>
         </is>
       </c>
       <c r="AD239" s="11" t="inlineStr">
@@ -33471,22 +33485,22 @@
       <c r="D240" s="10" t="inlineStr"/>
       <c r="E240" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>21.84</t>
         </is>
       </c>
       <c r="F240" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>18.84–24.25%</t>
         </is>
       </c>
       <c r="G240" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>&lt;LOQ</t>
         </is>
       </c>
       <c r="H240" s="9" t="inlineStr">
         <is>
-          <t>/</t>
+          <t>&lt;LOQ</t>
         </is>
       </c>
       <c r="I240" s="9" t="inlineStr">
@@ -33541,57 +33555,57 @@
       </c>
       <c r="S240" s="9" t="inlineStr">
         <is>
-          <t>2,5</t>
+          <t>/</t>
         </is>
       </c>
       <c r="T240" s="9" t="inlineStr">
         <is>
-          <t>н.д.</t>
+          <t>/</t>
         </is>
       </c>
       <c r="U240" s="9" t="inlineStr">
         <is>
-          <t>н.д.</t>
+          <t>/</t>
         </is>
       </c>
       <c r="V240" s="9" t="inlineStr">
         <is>
-          <t>н.д.</t>
+          <t>/</t>
         </is>
       </c>
       <c r="W240" s="9" t="inlineStr">
         <is>
-          <t>н.д.</t>
+          <t>/</t>
         </is>
       </c>
       <c r="X240" s="9" t="inlineStr">
         <is>
-          <t>н.д.</t>
+          <t>/</t>
         </is>
       </c>
       <c r="Y240" s="9" t="inlineStr">
         <is>
-          <t>н.д.</t>
+          <t>/</t>
         </is>
       </c>
       <c r="Z240" s="9" t="inlineStr">
         <is>
-          <t>н.д.</t>
+          <t>/</t>
         </is>
       </c>
       <c r="AA240" s="9" t="inlineStr">
         <is>
-          <t>1628-2026</t>
+          <t>100-3-K-26</t>
         </is>
       </c>
       <c r="AB240" s="9" t="inlineStr">
         <is>
-          <t>23.04.2026</t>
+          <t>09.04.2026</t>
         </is>
       </c>
       <c r="AC240" s="10" t="inlineStr">
         <is>
-          <t>IPH — Institute of Public Health (chemistry)</t>
+          <t>Farmahem</t>
         </is>
       </c>
       <c r="AD240" s="11" t="inlineStr">
@@ -33738,7 +33752,7 @@
     </row>
     <row r="242">
       <c r="A242" s="5" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B242" s="6" t="inlineStr">
         <is>
@@ -34568,7 +34582,7 @@
     </row>
     <row r="248">
       <c r="A248" s="5" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B248" s="6" t="inlineStr">
         <is>
@@ -34990,7 +35004,7 @@
     </row>
     <row r="251">
       <c r="A251" s="13" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B251" s="14" t="inlineStr">
         <is>
@@ -35412,7 +35426,7 @@
     </row>
     <row r="254">
       <c r="A254" s="5" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B254" s="6" t="inlineStr">
         <is>
@@ -35834,7 +35848,7 @@
     </row>
     <row r="257">
       <c r="A257" s="13" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B257" s="14" t="inlineStr">
         <is>
@@ -36248,7 +36262,7 @@
     </row>
     <row r="260">
       <c r="A260" s="5" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B260" s="6" t="inlineStr">
         <is>
@@ -36670,7 +36684,7 @@
     </row>
     <row r="263">
       <c r="A263" s="13" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B263" s="14" t="inlineStr">
         <is>
@@ -37084,7 +37098,7 @@
     </row>
     <row r="266">
       <c r="A266" s="5" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B266" s="6" t="inlineStr">
         <is>
@@ -37774,7 +37788,7 @@
     </row>
     <row r="271">
       <c r="A271" s="13" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B271" s="14" t="inlineStr">
         <is>
@@ -38188,7 +38202,7 @@
     </row>
     <row r="274">
       <c r="A274" s="5" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B274" s="6" t="inlineStr">
         <is>
@@ -38610,7 +38624,7 @@
     </row>
     <row r="277">
       <c r="A277" s="5" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B277" s="6" t="inlineStr">
         <is>
@@ -38756,7 +38770,7 @@
     </row>
     <row r="278">
       <c r="A278" s="5" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B278" s="6" t="inlineStr">
         <is>
@@ -38906,7 +38920,7 @@
     </row>
     <row r="279">
       <c r="A279" s="5" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B279" s="6" t="inlineStr">
         <is>
@@ -39328,7 +39342,7 @@
     </row>
     <row r="282">
       <c r="A282" s="5" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B282" s="6" t="inlineStr">
         <is>
@@ -39474,7 +39488,7 @@
     </row>
     <row r="283">
       <c r="A283" s="5" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B283" s="6" t="inlineStr">
         <is>
@@ -39620,7 +39634,7 @@
     </row>
     <row r="284">
       <c r="A284" s="5" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B284" s="6" t="inlineStr">
         <is>
@@ -39766,7 +39780,7 @@
     </row>
     <row r="285">
       <c r="A285" s="5" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B285" s="6" t="inlineStr">
         <is>
@@ -39916,7 +39930,7 @@
     </row>
     <row r="286">
       <c r="A286" s="5" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B286" s="6" t="inlineStr">
         <is>
@@ -40066,7 +40080,7 @@
     </row>
     <row r="287">
       <c r="A287" s="5" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B287" s="6" t="inlineStr">
         <is>
@@ -40216,7 +40230,7 @@
     </row>
     <row r="288">
       <c r="A288" s="5" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B288" s="6" t="inlineStr">
         <is>
@@ -40362,7 +40376,7 @@
     </row>
     <row r="289">
       <c r="A289" s="5" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B289" s="6" t="inlineStr">
         <is>
@@ -40508,7 +40522,7 @@
     </row>
     <row r="290">
       <c r="A290" s="5" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B290" s="6" t="inlineStr">
         <is>
@@ -40654,7 +40668,7 @@
     </row>
     <row r="291">
       <c r="A291" s="5" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B291" s="6" t="inlineStr">
         <is>
@@ -40940,7 +40954,7 @@
     </row>
     <row r="293">
       <c r="A293" s="5" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B293" s="6" t="inlineStr">
         <is>
@@ -41226,7 +41240,7 @@
     </row>
     <row r="295">
       <c r="A295" s="5" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B295" s="6" t="inlineStr">
         <is>
@@ -46319,7 +46333,7 @@
     <row r="108">
       <c r="A108" s="6" t="inlineStr">
         <is>
-          <t>Jokerz 31      3 batch(es)</t>
+          <t>Jokerz 31      4 batch(es)</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr"/>
@@ -46516,7 +46530,7 @@
       </c>
       <c r="B114" s="12" t="inlineStr">
         <is>
-          <t>J31122501</t>
+          <t>J31122501 (hand-trimmed)</t>
         </is>
       </c>
       <c r="C114" s="9" t="inlineStr">
@@ -46526,48 +46540,62 @@
       </c>
       <c r="D114" s="9" t="inlineStr">
         <is>
+          <t>19.84</t>
+        </is>
+      </c>
+      <c r="E114" s="9" t="inlineStr">
+        <is>
+          <t>18.84–24.25%</t>
+        </is>
+      </c>
+      <c r="F114" s="9" t="inlineStr">
+        <is>
+          <t>100-2-K-26</t>
+        </is>
+      </c>
+      <c r="G114" s="9" t="inlineStr">
+        <is>
+          <t>09.04.2026</t>
+        </is>
+      </c>
+      <c r="H114" s="10" t="inlineStr">
+        <is>
+          <t>Farmahem</t>
+        </is>
+      </c>
+      <c r="I114" s="11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="9" t="n">
+        <v>54</v>
+      </c>
+      <c r="B115" s="12" t="inlineStr">
+        <is>
+          <t>J31122501 (machine-trimmed)</t>
+        </is>
+      </c>
+      <c r="C115" s="9" t="inlineStr">
+        <is>
+          <t>P060262</t>
+        </is>
+      </c>
+      <c r="D115" s="9" t="inlineStr">
+        <is>
           <t>21.84</t>
         </is>
       </c>
-      <c r="E114" s="9" t="inlineStr">
-        <is>
-          <t>/</t>
-        </is>
-      </c>
-      <c r="F114" s="9" t="inlineStr">
+      <c r="E115" s="9" t="inlineStr">
+        <is>
+          <t>18.84–24.25%</t>
+        </is>
+      </c>
+      <c r="F115" s="9" t="inlineStr">
         <is>
           <t>100-3-K-26</t>
-        </is>
-      </c>
-      <c r="G114" s="9" t="inlineStr">
-        <is>
-          <t>09.04.2026</t>
-        </is>
-      </c>
-      <c r="H114" s="10" t="inlineStr">
-        <is>
-          <t>Farmahem</t>
-        </is>
-      </c>
-      <c r="I114" s="11" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="9" t="inlineStr"/>
-      <c r="B115" s="10" t="inlineStr"/>
-      <c r="C115" s="9" t="inlineStr"/>
-      <c r="D115" s="9" t="inlineStr">
-        <is>
-          <t>19.84</t>
-        </is>
-      </c>
-      <c r="E115" s="9" t="inlineStr"/>
-      <c r="F115" s="9" t="inlineStr">
-        <is>
-          <t>100-2-K-26</t>
         </is>
       </c>
       <c r="G115" s="9" t="inlineStr">
@@ -46603,7 +46631,7 @@
     </row>
     <row r="117">
       <c r="A117" s="9" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B117" s="12" t="inlineStr">
         <is>
@@ -46663,7 +46691,7 @@
     </row>
     <row r="119">
       <c r="A119" s="9" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B119" s="12" t="inlineStr">
         <is>
@@ -46739,7 +46767,7 @@
     </row>
     <row r="121">
       <c r="A121" s="9" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B121" s="12" t="inlineStr">
         <is>
@@ -46830,7 +46858,7 @@
     </row>
     <row r="124">
       <c r="A124" s="9" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B124" s="12" t="inlineStr">
         <is>
@@ -46902,7 +46930,7 @@
     </row>
     <row r="126">
       <c r="A126" s="9" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B126" s="12" t="inlineStr">
         <is>
@@ -46978,7 +47006,7 @@
     </row>
     <row r="128">
       <c r="A128" s="9" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B128" s="12" t="inlineStr">
         <is>
@@ -47085,7 +47113,7 @@
     </row>
     <row r="131">
       <c r="A131" s="9" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B131" s="12" t="inlineStr">
         <is>
@@ -47161,7 +47189,7 @@
     </row>
     <row r="133">
       <c r="A133" s="9" t="n">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B133" s="12" t="inlineStr">
         <is>
@@ -47237,7 +47265,7 @@
     </row>
     <row r="135">
       <c r="A135" s="9" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B135" s="12" t="inlineStr">
         <is>
@@ -47313,7 +47341,7 @@
     </row>
     <row r="137">
       <c r="A137" s="9" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B137" s="12" t="inlineStr">
         <is>
@@ -47358,7 +47386,7 @@
     </row>
     <row r="138">
       <c r="A138" s="9" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B138" s="12" t="inlineStr">
         <is>
@@ -47449,7 +47477,7 @@
     </row>
     <row r="141">
       <c r="A141" s="9" t="n">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B141" s="12" t="inlineStr">
         <is>
@@ -47525,7 +47553,7 @@
     </row>
     <row r="143">
       <c r="A143" s="9" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B143" s="12" t="inlineStr">
         <is>
@@ -47585,7 +47613,7 @@
     </row>
     <row r="145">
       <c r="A145" s="9" t="n">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B145" s="12" t="inlineStr">
         <is>
@@ -47707,7 +47735,7 @@
     </row>
     <row r="149">
       <c r="A149" s="9" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B149" s="12" t="inlineStr">
         <is>
@@ -47752,7 +47780,7 @@
     </row>
     <row r="150">
       <c r="A150" s="9" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B150" s="12" t="inlineStr">
         <is>
@@ -47793,7 +47821,7 @@
     </row>
     <row r="151">
       <c r="A151" s="9" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B151" s="12" t="inlineStr">
         <is>
@@ -47853,7 +47881,7 @@
     </row>
     <row r="153">
       <c r="A153" s="9" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B153" s="12" t="inlineStr">
         <is>
@@ -47929,7 +47957,7 @@
     </row>
     <row r="155">
       <c r="A155" s="9" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B155" s="12" t="inlineStr">
         <is>
@@ -47974,7 +48002,7 @@
     </row>
     <row r="156">
       <c r="A156" s="9" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B156" s="12" t="inlineStr">
         <is>
@@ -48034,7 +48062,7 @@
     </row>
     <row r="158">
       <c r="A158" s="9" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B158" s="12" t="inlineStr">
         <is>
@@ -48079,7 +48107,7 @@
     </row>
     <row r="159">
       <c r="A159" s="9" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B159" s="12" t="inlineStr">
         <is>
@@ -48170,7 +48198,7 @@
     </row>
     <row r="162">
       <c r="A162" s="9" t="n">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B162" s="12" t="inlineStr">
         <is>
@@ -48211,7 +48239,7 @@
     </row>
     <row r="163">
       <c r="A163" s="9" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B163" s="12" t="inlineStr">
         <is>
@@ -48252,7 +48280,7 @@
     </row>
     <row r="164">
       <c r="A164" s="9" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B164" s="12" t="inlineStr">
         <is>
@@ -48440,7 +48468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M82"/>
+  <dimension ref="A1:M83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -51753,7 +51781,7 @@
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>J31122501</t>
+          <t>J31122501 (hand-trimmed)</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
@@ -51818,57 +51846,57 @@
       </c>
       <c r="B58" s="10" t="inlineStr">
         <is>
-          <t>OPM122501</t>
+          <t>J31122501 (machine-trimmed)</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>P060242</t>
+          <t>P060262</t>
         </is>
       </c>
       <c r="D58" s="10" t="inlineStr">
         <is>
-          <t>Orange Punch Mimosa</t>
+          <t>Jokerz 31</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>7.91</t>
+          <t>21.84</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr">
         <is>
-          <t>197-19-K-26, 07.08.2026, FHM</t>
+          <t>100-3-K-26, 09.04.2026, FHM</t>
         </is>
       </c>
       <c r="G58" s="9" t="inlineStr">
         <is>
-          <t>Pot.-1</t>
+          <t>Pot.-2</t>
         </is>
       </c>
       <c r="H58" s="9" t="inlineStr">
         <is>
-          <t>8.00%</t>
+          <t>21.00%</t>
         </is>
       </c>
       <c r="I58" s="9" t="inlineStr">
         <is>
-          <t>± 0.54%</t>
+          <t>± 2.10%</t>
         </is>
       </c>
       <c r="J58" s="9" t="inlineStr">
         <is>
-          <t>7.46% – 8.54%</t>
+          <t>18.90% – 23.10%</t>
         </is>
       </c>
       <c r="K58" s="10" t="inlineStr">
         <is>
-          <t>Citrus Bloom</t>
+          <t>Jokerz 31</t>
         </is>
       </c>
       <c r="L58" s="9" t="inlineStr">
         <is>
-          <t>STEADY</t>
+          <t>CAYN</t>
         </is>
       </c>
       <c r="M58" s="9" t="inlineStr">
@@ -51883,27 +51911,27 @@
       </c>
       <c r="B59" s="10" t="inlineStr">
         <is>
-          <t>CC112501</t>
+          <t>OPM122501</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>P060272</t>
+          <t>P060242</t>
         </is>
       </c>
       <c r="D59" s="10" t="inlineStr">
         <is>
-          <t>Cash Cow</t>
+          <t>Orange Punch Mimosa</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>13.35</t>
+          <t>7.91</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t>ППК26068, 11.05.2026, CNP</t>
+          <t>197-19-K-26, 07.08.2026, FHM</t>
         </is>
       </c>
       <c r="G59" s="9" t="inlineStr">
@@ -51913,22 +51941,22 @@
       </c>
       <c r="H59" s="9" t="inlineStr">
         <is>
-          <t>13.50%</t>
+          <t>8.00%</t>
         </is>
       </c>
       <c r="I59" s="9" t="inlineStr">
         <is>
-          <t>± 1.34%</t>
+          <t>± 0.54%</t>
         </is>
       </c>
       <c r="J59" s="9" t="inlineStr">
         <is>
-          <t>12.16% – 14.84%</t>
+          <t>7.46% – 8.54%</t>
         </is>
       </c>
       <c r="K59" s="10" t="inlineStr">
         <is>
-          <t>Payday</t>
+          <t>Citrus Bloom</t>
         </is>
       </c>
       <c r="L59" s="9" t="inlineStr">
@@ -51948,47 +51976,59 @@
       </c>
       <c r="B60" s="10" t="inlineStr">
         <is>
-          <t>FB012601_1</t>
+          <t>CC112501</t>
         </is>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>P060322</t>
+          <t>P060272</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
         <is>
-          <t>Fat Bastard</t>
+          <t>Cash Cow</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>14.68</t>
+          <t>13.35</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr">
         <is>
-          <t>ППК26067, 11.05.2026, CNP</t>
+          <t>ППК26068, 11.05.2026, CNP</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">
         <is>
-          <t>Spec III</t>
+          <t>Pot.-1</t>
         </is>
       </c>
       <c r="H60" s="9" t="inlineStr">
         <is>
-          <t>16.5%</t>
-        </is>
-      </c>
-      <c r="I60" s="9" t="inlineStr"/>
+          <t>13.50%</t>
+        </is>
+      </c>
+      <c r="I60" s="9" t="inlineStr">
+        <is>
+          <t>± 1.34%</t>
+        </is>
+      </c>
       <c r="J60" s="9" t="inlineStr">
         <is>
-          <t>13.68–19.25%</t>
-        </is>
-      </c>
-      <c r="K60" s="10" t="inlineStr"/>
-      <c r="L60" s="9" t="inlineStr"/>
+          <t>12.16% – 14.84%</t>
+        </is>
+      </c>
+      <c r="K60" s="10" t="inlineStr">
+        <is>
+          <t>Payday</t>
+        </is>
+      </c>
+      <c r="L60" s="9" t="inlineStr">
+        <is>
+          <t>STEADY</t>
+        </is>
+      </c>
       <c r="M60" s="9" t="inlineStr">
         <is>
           <t>ДА | YES</t>
@@ -52001,12 +52041,12 @@
       </c>
       <c r="B61" s="10" t="inlineStr">
         <is>
-          <t>FB112501</t>
+          <t>FB012601_1</t>
         </is>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>P060292</t>
+          <t>P060322</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
@@ -52016,44 +52056,32 @@
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>16.69</t>
+          <t>14.68</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
-          <t>ППК26066, 11.05.2026, CNP</t>
+          <t>ППК26067, 11.05.2026, CNP</t>
         </is>
       </c>
       <c r="G61" s="9" t="inlineStr">
         <is>
-          <t>Pot.-1</t>
+          <t>Spec III</t>
         </is>
       </c>
       <c r="H61" s="9" t="inlineStr">
         <is>
-          <t>16.00%</t>
-        </is>
-      </c>
-      <c r="I61" s="9" t="inlineStr">
-        <is>
-          <t>± 1.54%</t>
-        </is>
-      </c>
+          <t>16.5%</t>
+        </is>
+      </c>
+      <c r="I61" s="9" t="inlineStr"/>
       <c r="J61" s="9" t="inlineStr">
         <is>
-          <t>14.46% – 17.54%</t>
-        </is>
-      </c>
-      <c r="K61" s="10" t="inlineStr">
-        <is>
-          <t>Fat Sofa</t>
-        </is>
-      </c>
-      <c r="L61" s="9" t="inlineStr">
-        <is>
-          <t>CAYN</t>
-        </is>
-      </c>
+          <t>13.68–19.25%</t>
+        </is>
+      </c>
+      <c r="K61" s="10" t="inlineStr"/>
+      <c r="L61" s="9" t="inlineStr"/>
       <c r="M61" s="9" t="inlineStr">
         <is>
           <t>ДА | YES</t>
@@ -52066,28 +52094,64 @@
       </c>
       <c r="B62" s="10" t="inlineStr">
         <is>
-          <t>GG012601*</t>
-        </is>
-      </c>
-      <c r="C62" s="9" t="inlineStr"/>
-      <c r="D62" s="10" t="inlineStr"/>
+          <t>FB112501</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>P060292</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>Fat Bastard</t>
+        </is>
+      </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>15.35</t>
+          <t>16.69</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
         <is>
-          <t>ППК26062, 11.05.2026, CNP</t>
-        </is>
-      </c>
-      <c r="G62" s="9" t="inlineStr"/>
-      <c r="H62" s="9" t="inlineStr"/>
-      <c r="I62" s="9" t="inlineStr"/>
-      <c r="J62" s="9" t="inlineStr"/>
-      <c r="K62" s="10" t="inlineStr"/>
-      <c r="L62" s="9" t="inlineStr"/>
-      <c r="M62" s="9" t="inlineStr"/>
+          <t>ППК26066, 11.05.2026, CNP</t>
+        </is>
+      </c>
+      <c r="G62" s="9" t="inlineStr">
+        <is>
+          <t>Pot.-1</t>
+        </is>
+      </c>
+      <c r="H62" s="9" t="inlineStr">
+        <is>
+          <t>16.00%</t>
+        </is>
+      </c>
+      <c r="I62" s="9" t="inlineStr">
+        <is>
+          <t>± 1.54%</t>
+        </is>
+      </c>
+      <c r="J62" s="9" t="inlineStr">
+        <is>
+          <t>14.46% – 17.54%</t>
+        </is>
+      </c>
+      <c r="K62" s="10" t="inlineStr">
+        <is>
+          <t>Fat Sofa</t>
+        </is>
+      </c>
+      <c r="L62" s="9" t="inlineStr">
+        <is>
+          <t>CAYN</t>
+        </is>
+      </c>
+      <c r="M62" s="9" t="inlineStr">
+        <is>
+          <t>ДА | YES</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="n">
@@ -52095,64 +52159,28 @@
       </c>
       <c r="B63" s="10" t="inlineStr">
         <is>
-          <t>GG112501</t>
-        </is>
-      </c>
-      <c r="C63" s="9" t="inlineStr">
-        <is>
-          <t>P060252</t>
-        </is>
-      </c>
-      <c r="D63" s="10" t="inlineStr">
-        <is>
-          <t>Gorilla Glue</t>
-        </is>
-      </c>
+          <t>GG012601*</t>
+        </is>
+      </c>
+      <c r="C63" s="9" t="inlineStr"/>
+      <c r="D63" s="10" t="inlineStr"/>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>17.94</t>
+          <t>15.35</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
-          <t>ППК26061, 11.05.2026, CNP</t>
-        </is>
-      </c>
-      <c r="G63" s="9" t="inlineStr">
-        <is>
-          <t>Pot.-2</t>
-        </is>
-      </c>
-      <c r="H63" s="9" t="inlineStr">
-        <is>
-          <t>17.50%</t>
-        </is>
-      </c>
-      <c r="I63" s="9" t="inlineStr">
-        <is>
-          <t>± 1.75%</t>
-        </is>
-      </c>
-      <c r="J63" s="9" t="inlineStr">
-        <is>
-          <t>15.75% – 19.25%</t>
-        </is>
-      </c>
-      <c r="K63" s="10" t="inlineStr">
-        <is>
-          <t>Cherry Chocolate</t>
-        </is>
-      </c>
-      <c r="L63" s="9" t="inlineStr">
-        <is>
-          <t>CAYN</t>
-        </is>
-      </c>
-      <c r="M63" s="9" t="inlineStr">
-        <is>
-          <t>ДА | YES</t>
-        </is>
-      </c>
+          <t>ППК26062, 11.05.2026, CNP</t>
+        </is>
+      </c>
+      <c r="G63" s="9" t="inlineStr"/>
+      <c r="H63" s="9" t="inlineStr"/>
+      <c r="I63" s="9" t="inlineStr"/>
+      <c r="J63" s="9" t="inlineStr"/>
+      <c r="K63" s="10" t="inlineStr"/>
+      <c r="L63" s="9" t="inlineStr"/>
+      <c r="M63" s="9" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="9" t="n">
@@ -52160,28 +52188,64 @@
       </c>
       <c r="B64" s="10" t="inlineStr">
         <is>
-          <t>JD012601*</t>
-        </is>
-      </c>
-      <c r="C64" s="9" t="inlineStr"/>
-      <c r="D64" s="10" t="inlineStr"/>
+          <t>GG112501</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="inlineStr">
+        <is>
+          <t>P060252</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>Gorilla Glue</t>
+        </is>
+      </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>18.16</t>
+          <t>17.94</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr">
         <is>
-          <t>ППК26064, 11.05.2026, CNP</t>
-        </is>
-      </c>
-      <c r="G64" s="9" t="inlineStr"/>
-      <c r="H64" s="9" t="inlineStr"/>
-      <c r="I64" s="9" t="inlineStr"/>
-      <c r="J64" s="9" t="inlineStr"/>
-      <c r="K64" s="10" t="inlineStr"/>
-      <c r="L64" s="9" t="inlineStr"/>
-      <c r="M64" s="9" t="inlineStr"/>
+          <t>ППК26061, 11.05.2026, CNP</t>
+        </is>
+      </c>
+      <c r="G64" s="9" t="inlineStr">
+        <is>
+          <t>Pot.-2</t>
+        </is>
+      </c>
+      <c r="H64" s="9" t="inlineStr">
+        <is>
+          <t>17.50%</t>
+        </is>
+      </c>
+      <c r="I64" s="9" t="inlineStr">
+        <is>
+          <t>± 1.75%</t>
+        </is>
+      </c>
+      <c r="J64" s="9" t="inlineStr">
+        <is>
+          <t>15.75% – 19.25%</t>
+        </is>
+      </c>
+      <c r="K64" s="10" t="inlineStr">
+        <is>
+          <t>Cherry Chocolate</t>
+        </is>
+      </c>
+      <c r="L64" s="9" t="inlineStr">
+        <is>
+          <t>CAYN</t>
+        </is>
+      </c>
+      <c r="M64" s="9" t="inlineStr">
+        <is>
+          <t>ДА | YES</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="n">
@@ -52189,60 +52253,28 @@
       </c>
       <c r="B65" s="10" t="inlineStr">
         <is>
-          <t>JD112501</t>
+          <t>JD012601*</t>
         </is>
       </c>
       <c r="C65" s="9" t="inlineStr"/>
-      <c r="D65" s="10" t="inlineStr">
-        <is>
-          <t>Jelly Donutz</t>
-        </is>
-      </c>
+      <c r="D65" s="10" t="inlineStr"/>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>20.32</t>
+          <t>18.16</t>
         </is>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
-          <t>197-15-K-26, 07.08.2026, FHM</t>
-        </is>
-      </c>
-      <c r="G65" s="9" t="inlineStr">
-        <is>
-          <t>Pot.-2</t>
-        </is>
-      </c>
-      <c r="H65" s="9" t="inlineStr">
-        <is>
-          <t>20.00%</t>
-        </is>
-      </c>
-      <c r="I65" s="9" t="inlineStr">
-        <is>
-          <t>± 2.00%</t>
-        </is>
-      </c>
-      <c r="J65" s="9" t="inlineStr">
-        <is>
-          <t>18.00% – 22.00%</t>
-        </is>
-      </c>
-      <c r="K65" s="10" t="inlineStr">
-        <is>
-          <t>Jelly Donuts</t>
-        </is>
-      </c>
-      <c r="L65" s="9" t="inlineStr">
-        <is>
-          <t>CAYN</t>
-        </is>
-      </c>
-      <c r="M65" s="9" t="inlineStr">
-        <is>
-          <t>ДА | YES</t>
-        </is>
-      </c>
+          <t>ППК26064, 11.05.2026, CNP</t>
+        </is>
+      </c>
+      <c r="G65" s="9" t="inlineStr"/>
+      <c r="H65" s="9" t="inlineStr"/>
+      <c r="I65" s="9" t="inlineStr"/>
+      <c r="J65" s="9" t="inlineStr"/>
+      <c r="K65" s="10" t="inlineStr"/>
+      <c r="L65" s="9" t="inlineStr"/>
+      <c r="M65" s="9" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="9" t="n">
@@ -52250,28 +52282,60 @@
       </c>
       <c r="B66" s="10" t="inlineStr">
         <is>
-          <t>JD112501*</t>
+          <t>JD112501</t>
         </is>
       </c>
       <c r="C66" s="9" t="inlineStr"/>
-      <c r="D66" s="10" t="inlineStr"/>
+      <c r="D66" s="10" t="inlineStr">
+        <is>
+          <t>Jelly Donutz</t>
+        </is>
+      </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>13.93</t>
+          <t>20.32</t>
         </is>
       </c>
       <c r="F66" s="10" t="inlineStr">
         <is>
-          <t>ППК26065, 11.05.2026, CNP</t>
-        </is>
-      </c>
-      <c r="G66" s="9" t="inlineStr"/>
-      <c r="H66" s="9" t="inlineStr"/>
-      <c r="I66" s="9" t="inlineStr"/>
-      <c r="J66" s="9" t="inlineStr"/>
-      <c r="K66" s="10" t="inlineStr"/>
-      <c r="L66" s="9" t="inlineStr"/>
-      <c r="M66" s="9" t="inlineStr"/>
+          <t>197-15-K-26, 07.08.2026, FHM</t>
+        </is>
+      </c>
+      <c r="G66" s="9" t="inlineStr">
+        <is>
+          <t>Pot.-2</t>
+        </is>
+      </c>
+      <c r="H66" s="9" t="inlineStr">
+        <is>
+          <t>20.00%</t>
+        </is>
+      </c>
+      <c r="I66" s="9" t="inlineStr">
+        <is>
+          <t>± 2.00%</t>
+        </is>
+      </c>
+      <c r="J66" s="9" t="inlineStr">
+        <is>
+          <t>18.00% – 22.00%</t>
+        </is>
+      </c>
+      <c r="K66" s="10" t="inlineStr">
+        <is>
+          <t>Jelly Donuts</t>
+        </is>
+      </c>
+      <c r="L66" s="9" t="inlineStr">
+        <is>
+          <t>CAYN</t>
+        </is>
+      </c>
+      <c r="M66" s="9" t="inlineStr">
+        <is>
+          <t>ДА | YES</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="n">
@@ -52279,64 +52343,28 @@
       </c>
       <c r="B67" s="10" t="inlineStr">
         <is>
-          <t>SCR112501</t>
-        </is>
-      </c>
-      <c r="C67" s="9" t="inlineStr">
-        <is>
-          <t>P060282</t>
-        </is>
-      </c>
-      <c r="D67" s="10" t="inlineStr">
-        <is>
-          <t>Scrambler</t>
-        </is>
-      </c>
+          <t>JD112501*</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr"/>
+      <c r="D67" s="10" t="inlineStr"/>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>17.13</t>
+          <t>13.93</t>
         </is>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
-          <t>ППК26069, 11.05.2026, CNP</t>
-        </is>
-      </c>
-      <c r="G67" s="9" t="inlineStr">
-        <is>
-          <t>Pot.-1</t>
-        </is>
-      </c>
-      <c r="H67" s="9" t="inlineStr">
-        <is>
-          <t>18.00%</t>
-        </is>
-      </c>
-      <c r="I67" s="9" t="inlineStr">
-        <is>
-          <t>± 1.79%</t>
-        </is>
-      </c>
-      <c r="J67" s="9" t="inlineStr">
-        <is>
-          <t>16.21% – 19.79%</t>
-        </is>
-      </c>
-      <c r="K67" s="10" t="inlineStr">
-        <is>
-          <t>Scrambler</t>
-        </is>
-      </c>
-      <c r="L67" s="9" t="inlineStr">
-        <is>
-          <t>CAYN</t>
-        </is>
-      </c>
-      <c r="M67" s="9" t="inlineStr">
-        <is>
-          <t>ДА | YES</t>
-        </is>
-      </c>
+          <t>ППК26065, 11.05.2026, CNP</t>
+        </is>
+      </c>
+      <c r="G67" s="9" t="inlineStr"/>
+      <c r="H67" s="9" t="inlineStr"/>
+      <c r="I67" s="9" t="inlineStr"/>
+      <c r="J67" s="9" t="inlineStr"/>
+      <c r="K67" s="10" t="inlineStr"/>
+      <c r="L67" s="9" t="inlineStr"/>
+      <c r="M67" s="9" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="9" t="n">
@@ -52344,48 +52372,52 @@
       </c>
       <c r="B68" s="10" t="inlineStr">
         <is>
-          <t>FB012603</t>
-        </is>
-      </c>
-      <c r="C68" s="9" t="inlineStr"/>
+          <t>SCR112501</t>
+        </is>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>P060282</t>
+        </is>
+      </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>Fat Bastard</t>
+          <t>Scrambler</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>20.83</t>
+          <t>17.13</t>
         </is>
       </c>
       <c r="F68" s="10" t="inlineStr">
         <is>
-          <t>ППК26112, 30.06.2026, CNP</t>
+          <t>ППК26069, 11.05.2026, CNP</t>
         </is>
       </c>
       <c r="G68" s="9" t="inlineStr">
         <is>
-          <t>Pot.-2</t>
+          <t>Pot.-1</t>
         </is>
       </c>
       <c r="H68" s="9" t="inlineStr">
         <is>
-          <t>19.50%</t>
+          <t>18.00%</t>
         </is>
       </c>
       <c r="I68" s="9" t="inlineStr">
         <is>
-          <t>± 1.95%</t>
+          <t>± 1.79%</t>
         </is>
       </c>
       <c r="J68" s="9" t="inlineStr">
         <is>
-          <t>17.55% – 21.45%</t>
+          <t>16.21% – 19.79%</t>
         </is>
       </c>
       <c r="K68" s="10" t="inlineStr">
         <is>
-          <t>Daywalker</t>
+          <t>Scrambler</t>
         </is>
       </c>
       <c r="L68" s="9" t="inlineStr">
@@ -52405,14 +52437,10 @@
       </c>
       <c r="B69" s="10" t="inlineStr">
         <is>
-          <t>FB012603V</t>
-        </is>
-      </c>
-      <c r="C69" s="9" t="inlineStr">
-        <is>
-          <t>P060392</t>
-        </is>
-      </c>
+          <t>FB012603</t>
+        </is>
+      </c>
+      <c r="C69" s="9" t="inlineStr"/>
       <c r="D69" s="10" t="inlineStr">
         <is>
           <t>Fat Bastard</t>
@@ -52420,12 +52448,12 @@
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>18.29</t>
+          <t>20.83</t>
         </is>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
-          <t>ППК26110, 30.06.2026, CNP</t>
+          <t>ППК26112, 30.06.2026, CNP</t>
         </is>
       </c>
       <c r="G69" s="9" t="inlineStr">
@@ -52470,27 +52498,27 @@
       </c>
       <c r="B70" s="10" t="inlineStr">
         <is>
-          <t>GG012603</t>
+          <t>FB012603V</t>
         </is>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>P060402</t>
+          <t>P060392</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>Gorilla Glue</t>
+          <t>Fat Bastard</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>16.70</t>
+          <t>18.29</t>
         </is>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t>197-8-K-26, 07.08.2026, FHM</t>
+          <t>ППК26110, 30.06.2026, CNP</t>
         </is>
       </c>
       <c r="G70" s="9" t="inlineStr">
@@ -52500,27 +52528,27 @@
       </c>
       <c r="H70" s="9" t="inlineStr">
         <is>
-          <t>17.50%</t>
+          <t>19.50%</t>
         </is>
       </c>
       <c r="I70" s="9" t="inlineStr">
         <is>
-          <t>± 1.75%</t>
+          <t>± 1.95%</t>
         </is>
       </c>
       <c r="J70" s="9" t="inlineStr">
         <is>
-          <t>15.75% – 19.25%</t>
+          <t>17.55% – 21.45%</t>
         </is>
       </c>
       <c r="K70" s="10" t="inlineStr">
         <is>
-          <t>GG4</t>
+          <t>Daywalker</t>
         </is>
       </c>
       <c r="L70" s="9" t="inlineStr">
         <is>
-          <t>STEADY</t>
+          <t>CAYN</t>
         </is>
       </c>
       <c r="M70" s="9" t="inlineStr">
@@ -52535,23 +52563,27 @@
       </c>
       <c r="B71" s="10" t="inlineStr">
         <is>
-          <t>JD012603_02</t>
-        </is>
-      </c>
-      <c r="C71" s="9" t="inlineStr"/>
+          <t>GG012603</t>
+        </is>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>P060402</t>
+        </is>
+      </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>JellyDonutz</t>
+          <t>Gorilla Glue</t>
         </is>
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>20.54</t>
+          <t>16.70</t>
         </is>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t>ППК26113, 30.06.2026, CNP</t>
+          <t>197-8-K-26, 07.08.2026, FHM</t>
         </is>
       </c>
       <c r="G71" s="9" t="inlineStr">
@@ -52561,27 +52593,27 @@
       </c>
       <c r="H71" s="9" t="inlineStr">
         <is>
-          <t>20.00%</t>
+          <t>17.50%</t>
         </is>
       </c>
       <c r="I71" s="9" t="inlineStr">
         <is>
-          <t>± 2.00%</t>
+          <t>± 1.75%</t>
         </is>
       </c>
       <c r="J71" s="9" t="inlineStr">
         <is>
-          <t>18.00% – 22.00%</t>
+          <t>15.75% – 19.25%</t>
         </is>
       </c>
       <c r="K71" s="10" t="inlineStr">
         <is>
-          <t>Jelly Donuts</t>
+          <t>GG4</t>
         </is>
       </c>
       <c r="L71" s="9" t="inlineStr">
         <is>
-          <t>CAYN</t>
+          <t>STEADY</t>
         </is>
       </c>
       <c r="M71" s="9" t="inlineStr">
@@ -52596,7 +52628,7 @@
       </c>
       <c r="B72" s="10" t="inlineStr">
         <is>
-          <t>JD012603_02V</t>
+          <t>JD012603_02</t>
         </is>
       </c>
       <c r="C72" s="9" t="inlineStr"/>
@@ -52607,32 +52639,32 @@
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>15.16</t>
+          <t>20.54</t>
         </is>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
-          <t>ППК26111, 30.06.2026, CNP</t>
+          <t>ППК26113, 30.06.2026, CNP</t>
         </is>
       </c>
       <c r="G72" s="9" t="inlineStr">
         <is>
-          <t>Pot.-1</t>
+          <t>Pot.-2</t>
         </is>
       </c>
       <c r="H72" s="9" t="inlineStr">
         <is>
-          <t>16.50%</t>
+          <t>20.00%</t>
         </is>
       </c>
       <c r="I72" s="9" t="inlineStr">
         <is>
-          <t>± 1.49%</t>
+          <t>± 2.00%</t>
         </is>
       </c>
       <c r="J72" s="9" t="inlineStr">
         <is>
-          <t>15.01% – 17.99%</t>
+          <t>18.00% – 22.00%</t>
         </is>
       </c>
       <c r="K72" s="10" t="inlineStr">
@@ -52657,44 +52689,60 @@
       </c>
       <c r="B73" s="10" t="inlineStr">
         <is>
-          <t>JD022601</t>
+          <t>JD012603_02V</t>
         </is>
       </c>
       <c r="C73" s="9" t="inlineStr"/>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>Jelly Donutz</t>
+          <t>JellyDonutz</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>18.58</t>
+          <t>15.16</t>
         </is>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t>ППК26115, 30.06.2026, CNP</t>
+          <t>ППК26111, 30.06.2026, CNP</t>
         </is>
       </c>
       <c r="G73" s="9" t="inlineStr">
         <is>
-          <t>нема | none</t>
+          <t>Pot.-1</t>
         </is>
       </c>
       <c r="H73" s="9" t="inlineStr">
         <is>
-          <t>не е во залихата Т1/Т2/Т3 | not in T1/T2/T3 stock</t>
-        </is>
-      </c>
-      <c r="I73" s="9" t="inlineStr"/>
-      <c r="J73" s="9" t="inlineStr"/>
+          <t>16.50%</t>
+        </is>
+      </c>
+      <c r="I73" s="9" t="inlineStr">
+        <is>
+          <t>± 1.49%</t>
+        </is>
+      </c>
+      <c r="J73" s="9" t="inlineStr">
+        <is>
+          <t>15.01% – 17.99%</t>
+        </is>
+      </c>
       <c r="K73" s="10" t="inlineStr">
         <is>
-          <t>— не е во мастерот | not in master</t>
-        </is>
-      </c>
-      <c r="L73" s="9" t="inlineStr"/>
-      <c r="M73" s="9" t="inlineStr"/>
+          <t>Jelly Donuts</t>
+        </is>
+      </c>
+      <c r="L73" s="9" t="inlineStr">
+        <is>
+          <t>CAYN</t>
+        </is>
+      </c>
+      <c r="M73" s="9" t="inlineStr">
+        <is>
+          <t>ДА | YES</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="9" t="n">
@@ -52702,27 +52750,23 @@
       </c>
       <c r="B74" s="10" t="inlineStr">
         <is>
-          <t>P160012</t>
-        </is>
-      </c>
-      <c r="C74" s="9" t="inlineStr">
-        <is>
-          <t>P160012</t>
-        </is>
-      </c>
+          <t>JD022601</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr"/>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>GrapePie</t>
+          <t>Jelly Donutz</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>26.32</t>
+          <t>18.58</t>
         </is>
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
-          <t>ППК26117, 06.07.2026, CNP</t>
+          <t>ППК26115, 30.06.2026, CNP</t>
         </is>
       </c>
       <c r="G74" s="9" t="inlineStr">
@@ -52751,12 +52795,12 @@
       </c>
       <c r="B75" s="10" t="inlineStr">
         <is>
-          <t>P160022</t>
+          <t>P160012</t>
         </is>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>P160022</t>
+          <t>P160012</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
@@ -52766,12 +52810,12 @@
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>25.72</t>
+          <t>26.32</t>
         </is>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
-          <t>ППК26118, 06.07.2026, CNP</t>
+          <t>ППК26117, 06.07.2026, CNP</t>
         </is>
       </c>
       <c r="G75" s="9" t="inlineStr">
@@ -52800,12 +52844,12 @@
       </c>
       <c r="B76" s="10" t="inlineStr">
         <is>
-          <t>P160032</t>
+          <t>P160022</t>
         </is>
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>P160032</t>
+          <t>P160022</t>
         </is>
       </c>
       <c r="D76" s="10" t="inlineStr">
@@ -52815,12 +52859,12 @@
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>24.78</t>
+          <t>25.72</t>
         </is>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
-          <t>ППК26119, 06.07.2026, CNP</t>
+          <t>ППК26118, 06.07.2026, CNP</t>
         </is>
       </c>
       <c r="G76" s="9" t="inlineStr">
@@ -52849,60 +52893,48 @@
       </c>
       <c r="B77" s="10" t="inlineStr">
         <is>
-          <t>SCR022601</t>
-        </is>
-      </c>
-      <c r="C77" s="9" t="inlineStr"/>
+          <t>P160032</t>
+        </is>
+      </c>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>P160032</t>
+        </is>
+      </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>Scrambler</t>
+          <t>GrapePie</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>21.92</t>
+          <t>24.78</t>
         </is>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
-          <t>ППК26116, 06.07.2026, CNP</t>
+          <t>ППК26119, 06.07.2026, CNP</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>Pot.-2</t>
+          <t>нема | none</t>
         </is>
       </c>
       <c r="H77" s="9" t="inlineStr">
         <is>
-          <t>22.00%</t>
-        </is>
-      </c>
-      <c r="I77" s="9" t="inlineStr">
-        <is>
-          <t>± 2.20%</t>
-        </is>
-      </c>
-      <c r="J77" s="9" t="inlineStr">
-        <is>
-          <t>19.80% – 24.20%</t>
-        </is>
-      </c>
+          <t>не е во залихата Т1/Т2/Т3 | not in T1/T2/T3 stock</t>
+        </is>
+      </c>
+      <c r="I77" s="9" t="inlineStr"/>
+      <c r="J77" s="9" t="inlineStr"/>
       <c r="K77" s="10" t="inlineStr">
         <is>
-          <t>Rainbow Sherbet</t>
-        </is>
-      </c>
-      <c r="L77" s="9" t="inlineStr">
-        <is>
-          <t>STEADY</t>
-        </is>
-      </c>
-      <c r="M77" s="9" t="inlineStr">
-        <is>
-          <t>ДА | YES</t>
-        </is>
-      </c>
+          <t>— не е во мастерот | not in master</t>
+        </is>
+      </c>
+      <c r="L77" s="9" t="inlineStr"/>
+      <c r="M77" s="9" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="9" t="n">
@@ -52910,44 +52942,60 @@
       </c>
       <c r="B78" s="10" t="inlineStr">
         <is>
-          <t>FB032601</t>
+          <t>SCR022601</t>
         </is>
       </c>
       <c r="C78" s="9" t="inlineStr"/>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>Fat Bastard</t>
+          <t>Scrambler</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>12.39</t>
+          <t>21.92</t>
         </is>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
-          <t>ППК26127, 21.07.2026, CNP</t>
+          <t>ППК26116, 06.07.2026, CNP</t>
         </is>
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>нема | none</t>
+          <t>Pot.-2</t>
         </is>
       </c>
       <c r="H78" s="9" t="inlineStr">
         <is>
-          <t>не е во залихата Т1/Т2/Т3 | not in T1/T2/T3 stock</t>
-        </is>
-      </c>
-      <c r="I78" s="9" t="inlineStr"/>
-      <c r="J78" s="9" t="inlineStr"/>
+          <t>22.00%</t>
+        </is>
+      </c>
+      <c r="I78" s="9" t="inlineStr">
+        <is>
+          <t>± 2.20%</t>
+        </is>
+      </c>
+      <c r="J78" s="9" t="inlineStr">
+        <is>
+          <t>19.80% – 24.20%</t>
+        </is>
+      </c>
       <c r="K78" s="10" t="inlineStr">
         <is>
-          <t>— не е во мастерот | not in master</t>
-        </is>
-      </c>
-      <c r="L78" s="9" t="inlineStr"/>
-      <c r="M78" s="9" t="inlineStr"/>
+          <t>Rainbow Sherbet</t>
+        </is>
+      </c>
+      <c r="L78" s="9" t="inlineStr">
+        <is>
+          <t>STEADY</t>
+        </is>
+      </c>
+      <c r="M78" s="9" t="inlineStr">
+        <is>
+          <t>ДА | YES</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="9" t="n">
@@ -52955,23 +53003,23 @@
       </c>
       <c r="B79" s="10" t="inlineStr">
         <is>
-          <t>GG032601</t>
+          <t>FB032601</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr"/>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>Gorilla Glue</t>
+          <t>Fat Bastard</t>
         </is>
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>18.98</t>
+          <t>12.39</t>
         </is>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
-          <t>ППК26128, 21.07.2026, CNP</t>
+          <t>ППК26127, 21.07.2026, CNP</t>
         </is>
       </c>
       <c r="G79" s="9" t="inlineStr">
@@ -53000,64 +53048,44 @@
       </c>
       <c r="B80" s="10" t="inlineStr">
         <is>
-          <t>CC012601/1</t>
-        </is>
-      </c>
-      <c r="C80" s="9" t="inlineStr">
-        <is>
-          <t>P060332</t>
-        </is>
-      </c>
+          <t>GG032601</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr"/>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>Cash Cow</t>
+          <t>Gorilla Glue</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>17.67</t>
+          <t>18.98</t>
         </is>
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
-          <t>197-6-K-26, 07.08.2026, FHM</t>
+          <t>ППК26128, 21.07.2026, CNP</t>
         </is>
       </c>
       <c r="G80" s="9" t="inlineStr">
         <is>
-          <t>Pot.-2</t>
+          <t>нема | none</t>
         </is>
       </c>
       <c r="H80" s="9" t="inlineStr">
         <is>
-          <t>16.50%</t>
-        </is>
-      </c>
-      <c r="I80" s="9" t="inlineStr">
-        <is>
-          <t>± 1.65%</t>
-        </is>
-      </c>
-      <c r="J80" s="9" t="inlineStr">
-        <is>
-          <t>14.85% – 18.15%</t>
-        </is>
-      </c>
+          <t>не е во залихата Т1/Т2/Т3 | not in T1/T2/T3 stock</t>
+        </is>
+      </c>
+      <c r="I80" s="9" t="inlineStr"/>
+      <c r="J80" s="9" t="inlineStr"/>
       <c r="K80" s="10" t="inlineStr">
         <is>
-          <t>Payday</t>
-        </is>
-      </c>
-      <c r="L80" s="9" t="inlineStr">
-        <is>
-          <t>STEADY</t>
-        </is>
-      </c>
-      <c r="M80" s="9" t="inlineStr">
-        <is>
-          <t>ДА | YES</t>
-        </is>
-      </c>
+          <t>— не е во мастерот | not in master</t>
+        </is>
+      </c>
+      <c r="L80" s="9" t="inlineStr"/>
+      <c r="M80" s="9" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="9" t="n">
@@ -53065,27 +53093,27 @@
       </c>
       <c r="B81" s="10" t="inlineStr">
         <is>
-          <t>FB012602</t>
+          <t>CC012601/1</t>
         </is>
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>P060352</t>
+          <t>P060332</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>Fat Bastard</t>
+          <t>Cash Cow</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>18.86</t>
+          <t>17.67</t>
         </is>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>197-7-K-26, 07.08.2026, FHM</t>
+          <t>197-6-K-26, 07.08.2026, FHM</t>
         </is>
       </c>
       <c r="G81" s="9" t="inlineStr">
@@ -53095,27 +53123,27 @@
       </c>
       <c r="H81" s="9" t="inlineStr">
         <is>
-          <t>19.50%</t>
+          <t>16.50%</t>
         </is>
       </c>
       <c r="I81" s="9" t="inlineStr">
         <is>
-          <t>± 1.95%</t>
+          <t>± 1.65%</t>
         </is>
       </c>
       <c r="J81" s="9" t="inlineStr">
         <is>
-          <t>17.55% – 21.45%</t>
+          <t>14.85% – 18.15%</t>
         </is>
       </c>
       <c r="K81" s="10" t="inlineStr">
         <is>
-          <t>Fat Sofa</t>
+          <t>Payday</t>
         </is>
       </c>
       <c r="L81" s="9" t="inlineStr">
         <is>
-          <t>CAYN</t>
+          <t>STEADY</t>
         </is>
       </c>
       <c r="M81" s="9" t="inlineStr">
@@ -53130,60 +53158,125 @@
       </c>
       <c r="B82" s="10" t="inlineStr">
         <is>
+          <t>FB012602</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>P060352</t>
+        </is>
+      </c>
+      <c r="D82" s="10" t="inlineStr">
+        <is>
+          <t>Fat Bastard</t>
+        </is>
+      </c>
+      <c r="E82" s="9" t="inlineStr">
+        <is>
+          <t>18.86</t>
+        </is>
+      </c>
+      <c r="F82" s="10" t="inlineStr">
+        <is>
+          <t>197-7-K-26, 07.08.2026, FHM</t>
+        </is>
+      </c>
+      <c r="G82" s="9" t="inlineStr">
+        <is>
+          <t>Pot.-2</t>
+        </is>
+      </c>
+      <c r="H82" s="9" t="inlineStr">
+        <is>
+          <t>19.50%</t>
+        </is>
+      </c>
+      <c r="I82" s="9" t="inlineStr">
+        <is>
+          <t>± 1.95%</t>
+        </is>
+      </c>
+      <c r="J82" s="9" t="inlineStr">
+        <is>
+          <t>17.55% – 21.45%</t>
+        </is>
+      </c>
+      <c r="K82" s="10" t="inlineStr">
+        <is>
+          <t>Fat Sofa</t>
+        </is>
+      </c>
+      <c r="L82" s="9" t="inlineStr">
+        <is>
+          <t>CAYN</t>
+        </is>
+      </c>
+      <c r="M82" s="9" t="inlineStr">
+        <is>
+          <t>ДА | YES</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="9" t="n">
+        <v>79</v>
+      </c>
+      <c r="B83" s="10" t="inlineStr">
+        <is>
           <t>SCR012603</t>
         </is>
       </c>
-      <c r="C82" s="9" t="inlineStr">
+      <c r="C83" s="9" t="inlineStr">
         <is>
           <t>P060382</t>
         </is>
       </c>
-      <c r="D82" s="10" t="inlineStr">
+      <c r="D83" s="10" t="inlineStr">
         <is>
           <t>Scrambler</t>
         </is>
       </c>
-      <c r="E82" s="9" t="inlineStr">
+      <c r="E83" s="9" t="inlineStr">
         <is>
           <t>17.84</t>
         </is>
       </c>
-      <c r="F82" s="10" t="inlineStr">
+      <c r="F83" s="10" t="inlineStr">
         <is>
           <t>197-21-K-26, 07.08.2026, FHM</t>
         </is>
       </c>
-      <c r="G82" s="9" t="inlineStr">
+      <c r="G83" s="9" t="inlineStr">
         <is>
           <t>Pot.-1</t>
         </is>
       </c>
-      <c r="H82" s="9" t="inlineStr">
+      <c r="H83" s="9" t="inlineStr">
         <is>
           <t>18.00%</t>
         </is>
       </c>
-      <c r="I82" s="9" t="inlineStr">
+      <c r="I83" s="9" t="inlineStr">
         <is>
           <t>± 1.79%</t>
         </is>
       </c>
-      <c r="J82" s="9" t="inlineStr">
+      <c r="J83" s="9" t="inlineStr">
         <is>
           <t>16.21% – 19.79%</t>
         </is>
       </c>
-      <c r="K82" s="10" t="inlineStr">
+      <c r="K83" s="10" t="inlineStr">
         <is>
           <t>Scrambler</t>
         </is>
       </c>
-      <c r="L82" s="9" t="inlineStr">
+      <c r="L83" s="9" t="inlineStr">
         <is>
           <t>CAYN</t>
         </is>
       </c>
-      <c r="M82" s="9" t="inlineStr">
+      <c r="M83" s="9" t="inlineStr">
         <is>
           <t>ДА | YES</t>
         </is>
@@ -55630,7 +55723,7 @@
       </c>
       <c r="I56" s="10" t="inlineStr">
         <is>
-          <t>J31112501 (?, 20.21%) | J31122501 (2025-12, 19.84%)</t>
+          <t>J31112501 (?, 20.21%) | J31122501 (hand-trimmed) (2025-12, 19.84%) | J31122501 (machine-trimmed) (2025-12, 21.84%)</t>
         </is>
       </c>
     </row>
@@ -58468,7 +58561,7 @@
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>ППК25117 printed THC total 1.58 vs own components 15.38 — VERIFY ON PAPER; ППК25154 printed 1.87 same class; BSS052501 sheet 20.47 — probably the NGP result but the NGP scan parses as garbage, read off paper; GP062501 PP cert prints 24.89 vs tranche sheet 22.89 — QC decision; J31112501 sheet 25.00 = the March 051-5-K-26 result (25.27, CF-77/26), stale — superseded by the April retest 100-1-K-26 (20.21); J31122501 sheet 21.77 ≈ the 100-3-K-26 trimmed-sample result (21.84, CF-153/26) while the register carries the hand-trimmed 100-2-K-26 (19.84, CF-151/26) — same-day dual-preparation results: QC to decide which preparation is CoQ-forming.</t>
+          <t>ППК25117 printed THC total 1.58 vs own components 15.38 — VERIFY ON PAPER; ППК25154 printed 1.87 same class; BSS052501 sheet 20.47 — probably the NGP result but the NGP scan parses as garbage, read off paper; GP062501 PP cert prints 24.89 vs tranche sheet 22.89 — QC decision; J31112501 sheet 25.00 = the March 051-5-K-26 result (25.27, CF-77/26), stale — superseded by the April retest 100-1-K-26 (20.21); J31122501 RESOLVED 27.08.2026: QC designated the trimmed preparation (100-3-K-26, 21.84) as CoQ-forming; hand-trimmed 19.84 (100-2-K-26) kept as experimental processing-mode comparison of the same batch; tranche sheet prints 21.77 — transcription slip of 21.84, correct the sheet.</t>
         </is>
       </c>
     </row>

</xml_diff>